<commit_message>
Treat hare-wallaby as its own species, not an "other" bucket
Renames species code hare_wallaby_other -> hare_wallaby (label
"Hare-wallaby") in SPECIES_TREE and the XLSForm; recompiles the XForm.
No data exists under the old code yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/track_ttd_survey.xlsx
+++ b/track_ttd_survey.xlsx
@@ -1215,12 +1215,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>hare_wallaby_other</t>
+          <t>hare_wallaby</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Macropod – Hare-wallaby – other</t>
+          <t>Macropod – Hare-wallaby</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>

<commit_message>
Field feedback: plain labels, walk type, end confirm, change species, v2 tweaks
From the Nyangumarta trip feedback (#2) and the V2 list (#1):
- Plain-language labels: "Kangaroo / wallaby", "Camel, cow & other feral",
  "Dirt colour" (labels only; stored codes unchanged).
- New required walk_type field (road / bush walk) on the end-of-walk sheet
  and in the XLSForm.
- End walk asks "End this walk?" in a sheet instead of needing a second tap.
- A recorded animal can be changed before Save (from the Seen chips or the
  end-of-walk list), keeping its time to detection and location; changing to
  an already-recorded species merges them, keeping the earlier time.
- Drop observer names from settings, the record and the form.
- New app icon: kangaroo tracks instead of paw prints.
- Bump the service-worker cache to v2; recompile the XForm.

Closes #1
Closes #2

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/track_ttd_survey.xlsx
+++ b/track_ttd_survey.xlsx
@@ -630,44 +630,54 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>observer_names</t>
+          <t>duration_seconds</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Observer names</t>
+          <t>Survey duration (seconds)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Total walk time from start to end of survey</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>. &gt;= 0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>duration_seconds</t>
+          <t>people_searching</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Survey duration (seconds)</t>
+          <t>Number of people searching</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Total walk time from start to end of survey</t>
+          <t>Can be fractional, e.g. 1.5 if someone joined partway</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -677,93 +687,83 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>. &gt;= 0</t>
+          <t>. &gt; 0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Must be more than 0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>select_one yes_no_choices</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>people_searching</t>
+          <t>recent_rain</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Number of people searching</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Can be fractional, e.g. 1.5 if someone joined partway</t>
+          <t>Recent rain?</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>yes</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>. &gt; 0</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Must be more than 0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>select_one yes_no_choices</t>
+          <t>select_one substrate_choices</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>recent_rain</t>
+          <t>substrate</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Recent rain?</t>
+          <t>Dirt colour</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>red</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>select_one substrate_choices</t>
+          <t>select_one walk_type_choices</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>substrate</t>
+          <t>walk_type</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Substrate</t>
+          <t>Road walk or bush walk?</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>yes</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>red</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1056,44 +1056,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>species_choices</t>
+          <t>walk_type_choices</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sand_goanna</t>
+          <t>road</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Goanna – Sand goanna (Wanggali)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>goanna</t>
+          <t>Road walk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>species_choices</t>
+          <t>walk_type_choices</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>small_goanna</t>
+          <t>bush</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Goanna – Small goanna (e.g. spiny-tailed, pygmy)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>goanna</t>
+          <t>Bush walk</t>
         </is>
       </c>
     </row>
@@ -1105,12 +1095,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>perentie</t>
+          <t>sand_goanna</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Goanna – Perentie</t>
+          <t>Goanna – Sand goanna (Wanggali)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1127,12 +1117,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>yellow_spotted_goanna</t>
+          <t>small_goanna</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goanna – Yellow-spotted goanna</t>
+          <t>Goanna – Small goanna (e.g. spiny-tailed, pygmy)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1149,12 +1139,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>large_goanna_unsure</t>
+          <t>perentie</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goanna – Large goanna – unsure</t>
+          <t>Goanna – Perentie</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1171,17 +1161,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>wallaby_unsure</t>
+          <t>yellow_spotted_goanna</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Macropod – Wallaby – unsure</t>
+          <t>Goanna – Yellow-spotted goanna</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>macropod</t>
+          <t>goanna</t>
         </is>
       </c>
     </row>
@@ -1193,17 +1183,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>spectacled_hare_wallaby</t>
+          <t>large_goanna_unsure</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Macropod – Spectacled hare-wallaby</t>
+          <t>Goanna – Large goanna – unsure</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>macropod</t>
+          <t>goanna</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1205,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>hare_wallaby</t>
+          <t>wallaby_unsure</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Macropod – Hare-wallaby</t>
+          <t>Kangaroo / wallaby – Wallaby – unsure</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1237,12 +1227,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>agile_wallaby</t>
+          <t>spectacled_hare_wallaby</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Macropod – Agile wallaby</t>
+          <t>Kangaroo / wallaby – Spectacled hare-wallaby</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1259,12 +1249,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>nailtail_wallaby</t>
+          <t>hare_wallaby</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Macropod – Northern nailtail wallaby</t>
+          <t>Kangaroo / wallaby – Hare-wallaby</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1281,12 +1271,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>euro</t>
+          <t>agile_wallaby</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Macropod – Euro</t>
+          <t>Kangaroo / wallaby – Agile wallaby</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1303,12 +1293,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>red_kangaroo</t>
+          <t>nailtail_wallaby</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Macropod – Red kangaroo</t>
+          <t>Kangaroo / wallaby – Northern nailtail wallaby</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1325,12 +1315,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>western_grey_kangaroo</t>
+          <t>euro</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Macropod – Western grey kangaroo</t>
+          <t>Kangaroo / wallaby – Euro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1347,12 +1337,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>kangaroo_unsure</t>
+          <t>red_kangaroo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Macropod – Kangaroo – unsure</t>
+          <t>Kangaroo / wallaby – Red kangaroo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1369,17 +1359,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bluetongue</t>
+          <t>western_grey_kangaroo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lizard – Blue-tongue</t>
+          <t>Kangaroo / wallaby – Western grey kangaroo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>lizard</t>
+          <t>macropod</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1381,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>dragon</t>
+          <t>kangaroo_unsure</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Lizard – Dragon</t>
+          <t>Kangaroo / wallaby – Kangaroo – unsure</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>lizard</t>
+          <t>macropod</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1403,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sand_slider</t>
+          <t>bluetongue</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lizard – Sand slider (Lerista)</t>
+          <t>Lizard – Blue-tongue</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1435,12 +1425,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>legless_lizard</t>
+          <t>dragon</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Lizard – Legless lizard</t>
+          <t>Lizard – Dragon</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1457,12 +1447,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>skink</t>
+          <t>sand_slider</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lizard – Skink</t>
+          <t>Lizard – Sand slider (Lerista)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1479,12 +1469,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>great_desert_skink</t>
+          <t>legless_lizard</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Lizard – Great Desert Skink</t>
+          <t>Lizard – Legless lizard</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1501,12 +1491,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>thorny_devil</t>
+          <t>skink</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lizard – Thorny devil</t>
+          <t>Lizard – Skink</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1523,12 +1513,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>other_lizard</t>
+          <t>great_desert_skink</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Lizard – Other lizard (describe)</t>
+          <t>Lizard – Great Desert Skink</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1545,17 +1535,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>cat</t>
+          <t>thorny_devil</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cat / dog / fox – Cat</t>
+          <t>Lizard – Thorny devil</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>cat_dog_fox</t>
+          <t>lizard</t>
         </is>
       </c>
     </row>
@@ -1567,17 +1557,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>dingo</t>
+          <t>other_lizard</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cat / dog / fox – Dingo / dog</t>
+          <t>Lizard – Other lizard (describe)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>cat_dog_fox</t>
+          <t>lizard</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1579,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>fox</t>
+          <t>cat</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cat / dog / fox – Fox</t>
+          <t>Cat / dog / fox – Cat</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1611,17 +1601,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>snake_unsure</t>
+          <t>dingo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Snake – Snake – unsure</t>
+          <t>Cat / dog / fox – Dingo / dog</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>snake</t>
+          <t>cat_dog_fox</t>
         </is>
       </c>
     </row>
@@ -1633,17 +1623,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>death_adder</t>
+          <t>fox</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Snake – Death adder</t>
+          <t>Cat / dog / fox – Fox</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>snake</t>
+          <t>cat_dog_fox</t>
         </is>
       </c>
     </row>
@@ -1655,12 +1645,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>king_brown</t>
+          <t>snake_unsure</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Snake – King brown</t>
+          <t>Snake – Snake – unsure</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1677,12 +1667,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>death_adder</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Snake – Python</t>
+          <t>Snake – Death adder</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1699,12 +1689,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>small_snake</t>
+          <t>king_brown</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Snake – Small snake</t>
+          <t>Snake – King brown</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1721,17 +1711,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>hopping_mouse</t>
+          <t>python</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Native mammal – Hopping mouse</t>
+          <t>Snake – Python</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>native_mammal</t>
+          <t>snake</t>
         </is>
       </c>
     </row>
@@ -1743,17 +1733,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>bilby</t>
+          <t>small_snake</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Native mammal – Bilby</t>
+          <t>Snake – Small snake</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>native_mammal</t>
+          <t>snake</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1755,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>small_mammal</t>
+          <t>hopping_mouse</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Native mammal – Small mammal (mouse / dunnart)</t>
+          <t>Native mammal – Hopping mouse</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1787,12 +1777,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mulgara</t>
+          <t>bilby</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Native mammal – Mulgara / Ampurta</t>
+          <t>Native mammal – Bilby</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1809,12 +1799,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>large_rat</t>
+          <t>small_mammal</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Native mammal – Large rat</t>
+          <t>Native mammal – Small mammal (mouse / dunnart)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1831,12 +1821,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>bandicoot</t>
+          <t>mulgara</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Native mammal – Bandicoot</t>
+          <t>Native mammal – Mulgara / Ampurta</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1853,12 +1843,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>bettong</t>
+          <t>large_rat</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Native mammal – Bettong</t>
+          <t>Native mammal – Large rat</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1875,12 +1865,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>quoll</t>
+          <t>bandicoot</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Native mammal – Quoll</t>
+          <t>Native mammal – Bandicoot</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1897,12 +1887,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>echidna</t>
+          <t>bettong</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Native mammal – Echidna</t>
+          <t>Native mammal – Bettong</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1919,12 +1909,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>possum</t>
+          <t>quoll</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Native mammal – Possum</t>
+          <t>Native mammal – Quoll</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1941,12 +1931,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>marsupial_mole</t>
+          <t>echidna</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Native mammal – Marsupial mole</t>
+          <t>Native mammal – Echidna</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1963,12 +1953,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>other_mammal</t>
+          <t>possum</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Native mammal – Other mammal (describe)</t>
+          <t>Native mammal – Possum</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1985,17 +1975,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>bustard</t>
+          <t>marsupial_mole</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bird – Bustard (turkey)</t>
+          <t>Native mammal – Marsupial mole</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>bird</t>
+          <t>native_mammal</t>
         </is>
       </c>
     </row>
@@ -2007,17 +1997,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>emu</t>
+          <t>other_mammal</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bird – Emu</t>
+          <t>Native mammal – Other mammal (describe)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>bird</t>
+          <t>native_mammal</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2019,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>curlew</t>
+          <t>bustard</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bird – Curlew</t>
+          <t>Bird – Bustard (turkey)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2051,12 +2041,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>quail</t>
+          <t>emu</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bird – Quail</t>
+          <t>Bird – Emu</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2073,12 +2063,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>walking_bird_other</t>
+          <t>curlew</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Bird – Walking bird – other</t>
+          <t>Bird – Curlew</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2095,12 +2085,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>hopping_bird_other</t>
+          <t>quail</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bird – Hopping bird – other</t>
+          <t>Bird – Quail</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2117,17 +2107,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>camel</t>
+          <t>walking_bird_other</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Feral herbivore – Camel</t>
+          <t>Bird – Walking bird – other</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>feral_herbivore</t>
+          <t>bird</t>
         </is>
       </c>
     </row>
@@ -2139,17 +2129,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>cow</t>
+          <t>hopping_bird_other</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Feral herbivore – Cow</t>
+          <t>Bird – Hopping bird – other</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>feral_herbivore</t>
+          <t>bird</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2151,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>donkey</t>
+          <t>camel</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Feral herbivore – Donkey</t>
+          <t>Camel, cow &amp; other feral – Camel</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2183,12 +2173,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>horse</t>
+          <t>cow</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Feral herbivore – Horse</t>
+          <t>Camel, cow &amp; other feral – Cow</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2205,12 +2195,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>goat</t>
+          <t>donkey</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Feral herbivore – Goat</t>
+          <t>Camel, cow &amp; other feral – Donkey</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2227,12 +2217,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>pig</t>
+          <t>horse</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Feral herbivore – Pig</t>
+          <t>Camel, cow &amp; other feral – Horse</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2249,12 +2239,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>rabbit</t>
+          <t>goat</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Feral herbivore – Rabbit</t>
+          <t>Camel, cow &amp; other feral – Goat</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2271,17 +2261,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>insect</t>
+          <t>pig</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Other – Insect / invertebrate</t>
+          <t>Camel, cow &amp; other feral – Pig</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>feral_herbivore</t>
         </is>
       </c>
     </row>
@@ -2293,17 +2283,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>unknown_tracks</t>
+          <t>rabbit</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Other – Unknown tracks</t>
+          <t>Camel, cow &amp; other feral – Rabbit</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>feral_herbivore</t>
         </is>
       </c>
     </row>
@@ -2315,15 +2305,59 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
+          <t>insect</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Other – Insect / invertebrate</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
           <t>other</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>species_choices</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>unknown_tracks</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Other – Unknown tracks</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>species_choices</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
         <is>
           <t>Other – Other (describe)</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>other</t>
         </is>

</xml_diff>